<commit_message>
Corrected Celsius capitalisation in input XLSX file.
Running Units_Abox.py now results in:
```
si:degreeCelsius a si:SISpecialNamedUnit ;
    si:hasSymbol "°C"^^xsd:string ;
    si:isUnitOfQtyKind si:TEMC ;
    skos:prefLabel "degree Celsius"@en,
        "degré Celsius"@fr .
```
</commit_message>
<xml_diff>
--- a/CUQ/_docs/Units_Prefixes.xlsx
+++ b/CUQ/_docs/Units_Prefixes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gregordudle/Developments/Semantic-SI/CUQ/_docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jh25\git\SI-Reference-Point-2023\CUQ\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E68CC5-1D04-414A-9C73-156567226BFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22FB8F1E-5673-4CA6-8B6A-FA47A570D8E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="2920" windowWidth="25500" windowHeight="14320" activeTab="4" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
   </bookViews>
   <sheets>
     <sheet name="Prefixes" sheetId="3" r:id="rId1"/>
@@ -288,9 +288,6 @@
     <t>C</t>
   </si>
   <si>
-    <t>degree celsius</t>
-  </si>
-  <si>
     <t>farad</t>
   </si>
   <si>
@@ -402,9 +399,6 @@
     <t>°C</t>
   </si>
   <si>
-    <t>degré celsius</t>
-  </si>
-  <si>
     <t>ARRN</t>
   </si>
   <si>
@@ -952,6 +946,12 @@
   </si>
   <si>
     <t>chaptre</t>
+  </si>
+  <si>
+    <t>degree Celsius</t>
+  </si>
+  <si>
+    <t>degré Celsius</t>
   </si>
 </sst>
 </file>
@@ -1318,12 +1318,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A359D5A-52A8-E54D-810F-2890E8F81F39}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="4" max="4" width="10.83203125" style="2"/>
+    <col min="4" max="4" width="10.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -1337,10 +1337,10 @@
         <v>18</v>
       </c>
       <c r="E1" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -1354,7 +1354,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -1382,12 +1382,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C5" s="1">
         <v>1E+21</v>
@@ -1396,7 +1396,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -1410,7 +1410,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1424,7 +1424,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>36</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -1466,7 +1466,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1480,7 +1480,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -1494,7 +1494,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>44</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -1522,7 +1522,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>48</v>
       </c>
@@ -1536,7 +1536,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>50</v>
       </c>
@@ -1550,7 +1550,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>52</v>
       </c>
@@ -1561,13 +1561,13 @@
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="E17" t="s">
         <v>258</v>
       </c>
-      <c r="E17" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>53</v>
       </c>
@@ -1581,12 +1581,12 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B19" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C19" s="1">
         <v>9.9999999999999998E-13</v>
@@ -1595,7 +1595,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>56</v>
       </c>
@@ -1609,7 +1609,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>58</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>62</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>66</v>
       </c>
@@ -1687,19 +1687,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DE8A68B-8B60-3949-B0A8-4A96CE4D68DA}">
   <dimension ref="A1:L19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.35546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="79.33203125" customWidth="1"/>
-    <col min="7" max="7" width="42.33203125" customWidth="1"/>
-    <col min="8" max="8" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.35546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="79.35546875" customWidth="1"/>
+    <col min="7" max="7" width="42.35546875" customWidth="1"/>
+    <col min="8" max="8" width="19.640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -1734,154 +1734,154 @@
         <v>77</v>
       </c>
       <c r="L1" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>70</v>
       </c>
       <c r="F2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="G2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="K2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="L2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>70</v>
       </c>
       <c r="E3"/>
       <c r="F3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="G3" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H3" t="s">
         <v>14</v>
       </c>
       <c r="I3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J3" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K3" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="L3" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>71</v>
       </c>
       <c r="F4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="G4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H4" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="K4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="L4" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>70</v>
       </c>
       <c r="E5"/>
       <c r="F5" t="s">
+        <v>253</v>
+      </c>
+      <c r="G5" t="s">
         <v>255</v>
-      </c>
-      <c r="G5" t="s">
-        <v>257</v>
       </c>
       <c r="H5" t="s">
         <v>14</v>
       </c>
       <c r="I5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="J5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="L5" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>69</v>
@@ -1890,358 +1890,358 @@
         <v>71</v>
       </c>
       <c r="F6" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="G6" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="K6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="L6" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>70</v>
       </c>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="G7" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="H7" t="s">
         <v>14</v>
       </c>
       <c r="I7" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K7" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="L7" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B8" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C8" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>71</v>
       </c>
       <c r="F8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="G8" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="K8" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="L8" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B9" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>70</v>
       </c>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="G9" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H9" t="s">
         <v>14</v>
       </c>
       <c r="I9" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="L9" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>181</v>
+      </c>
+      <c r="B10" t="s">
+        <v>180</v>
+      </c>
+      <c r="C10" t="s">
+        <v>181</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="F10" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="G10" t="s">
+        <v>206</v>
+      </c>
+      <c r="H10" t="s">
+        <v>193</v>
+      </c>
+      <c r="K10" t="s">
+        <v>214</v>
+      </c>
+      <c r="L10" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
         <v>183</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>182</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>183</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="F10" t="s">
-        <v>266</v>
-      </c>
-      <c r="G10" t="s">
-        <v>208</v>
-      </c>
-      <c r="H10" t="s">
-        <v>195</v>
-      </c>
-      <c r="K10" t="s">
-        <v>216</v>
-      </c>
-      <c r="L10" t="s">
+      <c r="F11" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="G11" t="s">
+        <v>235</v>
+      </c>
+      <c r="H11" t="s">
+        <v>194</v>
+      </c>
+      <c r="K11" t="s">
+        <v>214</v>
+      </c>
+      <c r="L11" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
         <v>185</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>184</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C12" t="s">
         <v>185</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="F11" t="s">
-        <v>265</v>
-      </c>
-      <c r="G11" t="s">
-        <v>237</v>
-      </c>
-      <c r="H11" t="s">
-        <v>196</v>
-      </c>
-      <c r="K11" t="s">
-        <v>216</v>
-      </c>
-      <c r="L11" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>187</v>
-      </c>
-      <c r="B12" t="s">
-        <v>186</v>
-      </c>
-      <c r="C12" t="s">
-        <v>187</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>68</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F12" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="G12" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H12" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="K12" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="L12" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B13" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C13" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>71</v>
       </c>
       <c r="F13" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="G13" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="H13" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="K13" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="L13" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B14" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>70</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="G14" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="H14" t="s">
         <v>14</v>
       </c>
       <c r="I14" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="J14" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="K14" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="L14" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B15" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C15" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>71</v>
       </c>
       <c r="F15" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G15" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H15" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K15" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L15" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B16" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C16" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>70</v>
       </c>
       <c r="E16"/>
       <c r="F16" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="G16" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H16" t="s">
         <v>14</v>
       </c>
       <c r="I16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J16" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="K16" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="L16" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -2255,22 +2255,22 @@
         <v>68</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F17" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H17" t="s">
         <v>7</v>
       </c>
       <c r="K17" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="L17" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -2287,22 +2287,22 @@
         <v>71</v>
       </c>
       <c r="F18" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="G18" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
       </c>
       <c r="K18" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="L18" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -2317,25 +2317,25 @@
       </c>
       <c r="E19"/>
       <c r="F19" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="G19" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H19" t="s">
         <v>14</v>
       </c>
       <c r="I19" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="J19" t="s">
         <v>16</v>
       </c>
       <c r="K19" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="L19" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -2346,9 +2346,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EF3A1C2-6A3C-474E-908C-FA60BE09F193}">
   <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -2359,171 +2359,171 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C2" t="s">
+        <v>218</v>
+      </c>
+      <c r="D2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E2" t="s">
+        <v>142</v>
+      </c>
+      <c r="F2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C3" t="s">
+        <v>219</v>
+      </c>
+      <c r="D3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E3" t="s">
+        <v>144</v>
+      </c>
+      <c r="F3" t="s">
+        <v>169</v>
+      </c>
+      <c r="G3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
         <v>220</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C4" t="s">
+        <v>220</v>
+      </c>
+      <c r="D4" t="s">
+        <v>212</v>
+      </c>
+      <c r="E4" t="s">
+        <v>208</v>
+      </c>
+      <c r="F4" t="s">
+        <v>171</v>
+      </c>
+      <c r="G4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>221</v>
+      </c>
+      <c r="B5" t="s">
+        <v>226</v>
+      </c>
+      <c r="C5" t="s">
+        <v>221</v>
+      </c>
+      <c r="D5" t="s">
+        <v>213</v>
+      </c>
+      <c r="E5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F5" t="s">
+        <v>179</v>
+      </c>
+      <c r="G5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>222</v>
+      </c>
+      <c r="B6" t="s">
         <v>227</v>
       </c>
-      <c r="C2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D2" t="s">
-        <v>212</v>
-      </c>
-      <c r="E2" t="s">
-        <v>144</v>
-      </c>
-      <c r="F2" t="s">
-        <v>168</v>
-      </c>
-      <c r="G2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>221</v>
-      </c>
-      <c r="B3" t="s">
-        <v>221</v>
-      </c>
-      <c r="C3" t="s">
-        <v>221</v>
-      </c>
-      <c r="D3" t="s">
-        <v>213</v>
-      </c>
-      <c r="E3" t="s">
-        <v>146</v>
-      </c>
-      <c r="F3" t="s">
-        <v>171</v>
-      </c>
-      <c r="G3" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="C6" t="s">
         <v>222</v>
       </c>
-      <c r="B4" t="s">
-        <v>222</v>
-      </c>
-      <c r="C4" t="s">
-        <v>222</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="D6" t="s">
         <v>214</v>
-      </c>
-      <c r="E4" t="s">
-        <v>210</v>
-      </c>
-      <c r="F4" t="s">
-        <v>173</v>
-      </c>
-      <c r="G4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>223</v>
-      </c>
-      <c r="B5" t="s">
-        <v>228</v>
-      </c>
-      <c r="C5" t="s">
-        <v>223</v>
-      </c>
-      <c r="D5" t="s">
-        <v>215</v>
-      </c>
-      <c r="E5" t="s">
-        <v>149</v>
-      </c>
-      <c r="F5" t="s">
-        <v>181</v>
-      </c>
-      <c r="G5" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>224</v>
-      </c>
-      <c r="B6" t="s">
-        <v>229</v>
-      </c>
-      <c r="C6" t="s">
-        <v>224</v>
-      </c>
-      <c r="D6" t="s">
-        <v>216</v>
       </c>
       <c r="E6" t="s">
         <v>51</v>
       </c>
       <c r="F6" t="s">
+        <v>181</v>
+      </c>
+      <c r="G6" t="s">
         <v>183</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>185</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>187</v>
       </c>
-      <c r="I6" t="s">
-        <v>189</v>
-      </c>
       <c r="J6" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B7" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C7" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D7" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E7" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G7" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B8" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D8" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E8" t="s">
         <v>19</v>
@@ -2546,12 +2546,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{837449F3-3B63-3745-8303-091E9EC09344}">
   <dimension ref="A1:E23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="4" max="4" width="10.83203125" style="2"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -2568,7 +2569,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -2582,10 +2583,10 @@
         <v>79</v>
       </c>
       <c r="E2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -2599,347 +2600,347 @@
         <v>81</v>
       </c>
       <c r="E3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B4" t="s">
+        <v>303</v>
+      </c>
+      <c r="C4" t="s">
+        <v>302</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>143</v>
-      </c>
-      <c r="B4" t="s">
-        <v>120</v>
-      </c>
-      <c r="C4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E4" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E5" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B6" t="s">
-        <v>85</v>
-      </c>
-      <c r="C6" t="s">
-        <v>85</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E6" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E8" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" t="s">
-        <v>87</v>
-      </c>
-      <c r="C7" t="s">
-        <v>87</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E7" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E9" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B8" t="s">
-        <v>89</v>
-      </c>
-      <c r="C8" t="s">
-        <v>89</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E8" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>92</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E10" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>91</v>
-      </c>
-      <c r="B9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="E9" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" t="s">
+        <v>94</v>
+      </c>
+      <c r="C11" t="s">
+        <v>94</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E11" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>93</v>
-      </c>
-      <c r="B10" t="s">
-        <v>93</v>
-      </c>
-      <c r="C10" t="s">
-        <v>93</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="E10" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>96</v>
+      </c>
+      <c r="C12" t="s">
+        <v>96</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E12" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>95</v>
-      </c>
-      <c r="B11" t="s">
-        <v>95</v>
-      </c>
-      <c r="C11" t="s">
-        <v>95</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="E11" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C13" t="s">
+        <v>98</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>97</v>
-      </c>
-      <c r="B12" t="s">
-        <v>97</v>
-      </c>
-      <c r="C12" t="s">
-        <v>97</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E12" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" t="s">
+        <v>100</v>
+      </c>
+      <c r="C14" t="s">
+        <v>100</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="E14" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>99</v>
-      </c>
-      <c r="B13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C13" t="s">
-        <v>99</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="E13" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" t="s">
+        <v>101</v>
+      </c>
+      <c r="C15" t="s">
+        <v>101</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E15" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>101</v>
-      </c>
-      <c r="B14" t="s">
-        <v>101</v>
-      </c>
-      <c r="C14" t="s">
-        <v>101</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="E14" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16" t="s">
+        <v>103</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E16" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>102</v>
-      </c>
-      <c r="B15" t="s">
-        <v>102</v>
-      </c>
-      <c r="C15" t="s">
-        <v>102</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E15" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>105</v>
+      </c>
+      <c r="B17" t="s">
+        <v>105</v>
+      </c>
+      <c r="C17" t="s">
+        <v>105</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E17" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>104</v>
-      </c>
-      <c r="B16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" t="s">
-        <v>104</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E16" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" t="s">
+        <v>107</v>
+      </c>
+      <c r="C18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E18" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>106</v>
-      </c>
-      <c r="B17" t="s">
-        <v>106</v>
-      </c>
-      <c r="C17" t="s">
-        <v>106</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E17" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" t="s">
+        <v>109</v>
+      </c>
+      <c r="C19" t="s">
+        <v>109</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>108</v>
-      </c>
-      <c r="B18" t="s">
-        <v>108</v>
-      </c>
-      <c r="C18" t="s">
-        <v>108</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E18" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>110</v>
-      </c>
-      <c r="B19" t="s">
-        <v>110</v>
-      </c>
-      <c r="C19" t="s">
-        <v>110</v>
-      </c>
-      <c r="D19" s="2" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
         <v>111</v>
       </c>
-      <c r="E19" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>112</v>
-      </c>
       <c r="B20" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C20" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>35</v>
       </c>
       <c r="E20" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21" t="s">
+        <v>112</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E21" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>114</v>
+      </c>
+      <c r="B22" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" t="s">
+        <v>114</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E22" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>113</v>
-      </c>
-      <c r="B21" t="s">
-        <v>113</v>
-      </c>
-      <c r="C21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="E21" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>116</v>
+      </c>
+      <c r="B23" t="s">
+        <v>116</v>
+      </c>
+      <c r="C23" t="s">
+        <v>116</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E23" t="s">
         <v>140</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>115</v>
-      </c>
-      <c r="B22" t="s">
-        <v>115</v>
-      </c>
-      <c r="C22" t="s">
-        <v>115</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E22" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>117</v>
-      </c>
-      <c r="B23" t="s">
-        <v>117</v>
-      </c>
-      <c r="C23" t="s">
-        <v>117</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E23" t="s">
-        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -2950,42 +2951,42 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC3BD8C3-F79C-5947-ABF9-F73A9D2E6571}">
   <dimension ref="A2:K27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="21.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" customWidth="1"/>
-    <col min="4" max="5" width="14.1640625" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+    <col min="1" max="1" width="21.85546875" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.640625" customWidth="1"/>
+    <col min="4" max="5" width="14.140625" customWidth="1"/>
+    <col min="6" max="6" width="20.35546875" customWidth="1"/>
+    <col min="10" max="10" width="25.85546875" customWidth="1"/>
     <col min="11" max="11" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B2" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
         <v>300</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>302</v>
       </c>
       <c r="B3">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -3002,302 +3003,302 @@
         <v>77</v>
       </c>
       <c r="F6" t="s">
+        <v>267</v>
+      </c>
+      <c r="G6" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>268</v>
+      </c>
+      <c r="B7" t="s">
+        <v>268</v>
+      </c>
+      <c r="C7" t="s">
+        <v>268</v>
+      </c>
+      <c r="D7" t="s">
         <v>269</v>
       </c>
-      <c r="G6" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>270</v>
-      </c>
-      <c r="B7" t="s">
-        <v>270</v>
-      </c>
-      <c r="C7" t="s">
-        <v>270</v>
-      </c>
-      <c r="D7" t="s">
-        <v>271</v>
-      </c>
       <c r="E7" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F7">
         <v>60</v>
       </c>
       <c r="G7" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C8" t="s">
         <v>272</v>
-      </c>
-      <c r="C8" t="s">
-        <v>274</v>
       </c>
       <c r="D8" t="s">
         <v>43</v>
       </c>
       <c r="E8" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F8">
         <v>3600</v>
       </c>
       <c r="G8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B9" t="s">
+        <v>271</v>
+      </c>
+      <c r="C9" t="s">
         <v>273</v>
-      </c>
-      <c r="C9" t="s">
-        <v>275</v>
       </c>
       <c r="D9" t="s">
         <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F9">
         <v>86400</v>
       </c>
       <c r="G9" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
+        <v>274</v>
+      </c>
+      <c r="B10" t="s">
+        <v>289</v>
+      </c>
+      <c r="C10" t="s">
+        <v>275</v>
+      </c>
+      <c r="D10" t="s">
         <v>276</v>
       </c>
-      <c r="B10" t="s">
-        <v>291</v>
-      </c>
-      <c r="C10" t="s">
-        <v>277</v>
-      </c>
-      <c r="D10" t="s">
-        <v>278</v>
-      </c>
       <c r="E10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F10" s="7">
         <v>149597870700</v>
       </c>
       <c r="G10" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B11" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C11" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E11" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F11" s="5">
         <v>1.7453292519943299E-2</v>
       </c>
       <c r="G11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H11">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B12" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C12" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="E12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F12" s="5">
         <v>2.9088820866572201E-4</v>
       </c>
       <c r="G12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B13" t="s">
+        <v>294</v>
+      </c>
+      <c r="C13" t="s">
+        <v>293</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="C13" t="s">
-        <v>295</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>298</v>
-      </c>
       <c r="E13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F13" s="5">
         <v>4.8481368110953598E-6</v>
       </c>
       <c r="G13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
+        <v>279</v>
+      </c>
+      <c r="B14" t="s">
+        <v>279</v>
+      </c>
+      <c r="C14" t="s">
+        <v>279</v>
+      </c>
+      <c r="D14" t="s">
+        <v>280</v>
+      </c>
+      <c r="E14" t="s">
         <v>281</v>
-      </c>
-      <c r="B14" t="s">
-        <v>281</v>
-      </c>
-      <c r="C14" t="s">
-        <v>281</v>
-      </c>
-      <c r="D14" t="s">
-        <v>282</v>
-      </c>
-      <c r="E14" t="s">
-        <v>283</v>
       </c>
       <c r="F14">
         <v>1E-3</v>
       </c>
       <c r="G14" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H14">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D15" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E15" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F15">
         <v>1000</v>
       </c>
       <c r="G15" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H15">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B16" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C16" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D16" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E16" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F16" s="6">
         <v>1.6605390666E-27</v>
       </c>
       <c r="G16" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H16">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B17" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C17" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D17" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E17" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F17" s="7">
         <v>1.6021766339999999E-19</v>
       </c>
       <c r="G17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H17">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
       <c r="K25" s="4"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
       <c r="J27" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SI-Reference-Point-2023-12 units.ttl : stéradian (FR)
Fix for the French name of stéradian...
</commit_message>
<xml_diff>
--- a/CUQ/_docs/Units_Prefixes.xlsx
+++ b/CUQ/_docs/Units_Prefixes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10910"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n00002621/PycharmProjects/SI-Reference-Point-2023/CUQ/_docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B130A1-8333-2C43-A339-169CA1301B8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{338CB9CF-E79E-FC45-BDF2-3221ACA5401B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2140" yWindow="1900" windowWidth="55260" windowHeight="20480" activeTab="3" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
+    <workbookView xWindow="13620" yWindow="8420" windowWidth="55260" windowHeight="20480" activeTab="3" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
   </bookViews>
   <sheets>
     <sheet name="Prefixes" sheetId="3" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="SIUnitsSpecialNames" sheetId="4" r:id="rId4"/>
     <sheet name="NonSIUnits" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="404">
   <si>
     <t>hasStartValidity</t>
   </si>
@@ -1303,6 +1303,9 @@
   </si>
   <si>
     <t>℃</t>
+  </si>
+  <si>
+    <t>stéradian</t>
   </si>
 </sst>
 </file>
@@ -3662,7 +3665,7 @@
         <v>107</v>
       </c>
       <c r="B19" t="s">
-        <v>107</v>
+        <v>403</v>
       </c>
       <c r="C19" t="s">
         <v>107</v>

</xml_diff>

<commit_message>
fix typos in the excel files
</commit_message>
<xml_diff>
--- a/CUQ/_docs/Units_Prefixes.xlsx
+++ b/CUQ/_docs/Units_Prefixes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gruber04\git_repos\BIPM\Semantic-SI\CUQ\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0387F7-7D82-4620-AEFA-D53152158CEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C277D10A-8DA3-4677-BD4A-F0063F24151F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-8310" windowWidth="38640" windowHeight="21390" activeTab="1" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
+    <workbookView xWindow="28680" yWindow="-8310" windowWidth="38640" windowHeight="21390" activeTab="4" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
   </bookViews>
   <sheets>
     <sheet name="Prefixes" sheetId="3" r:id="rId1"/>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="403">
   <si>
     <t>hasStartValidity</t>
   </si>
@@ -918,9 +918,6 @@
     <t>dalton</t>
   </si>
   <si>
-    <t>electrovolt</t>
-  </si>
-  <si>
     <t>eV</t>
   </si>
   <si>
@@ -966,9 +963,6 @@
     <t>edition</t>
   </si>
   <si>
-    <t>chaptre</t>
-  </si>
-  <si>
     <t>degree Celsius</t>
   </si>
   <si>
@@ -1306,6 +1300,9 @@
   </si>
   <si>
     <t>stéradian</t>
+  </si>
+  <si>
+    <t>chapter</t>
   </si>
 </sst>
 </file>
@@ -1760,7 +1757,7 @@
         <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1780,7 +1777,7 @@
         <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1800,7 +1797,7 @@
         <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1820,7 +1817,7 @@
         <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1840,7 +1837,7 @@
         <v>29</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1851,7 +1848,7 @@
         <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="D7" s="1">
         <v>1000000000000000</v>
@@ -1860,7 +1857,7 @@
         <v>31</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1871,7 +1868,7 @@
         <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D8" s="1">
         <v>1000000000000</v>
@@ -1880,7 +1877,7 @@
         <v>33</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1900,7 +1897,7 @@
         <v>35</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1911,7 +1908,7 @@
         <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="D10" s="1">
         <v>1000000</v>
@@ -1920,7 +1917,7 @@
         <v>37</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1940,7 +1937,7 @@
         <v>39</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1960,7 +1957,7 @@
         <v>41</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1971,7 +1968,7 @@
         <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D13" s="1">
         <v>10</v>
@@ -1980,7 +1977,7 @@
         <v>43</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1991,7 +1988,7 @@
         <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="D14" s="1">
         <v>0.1</v>
@@ -2000,7 +1997,7 @@
         <v>45</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -2020,7 +2017,7 @@
         <v>47</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -2040,7 +2037,7 @@
         <v>49</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2060,7 +2057,7 @@
         <v>246</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="G17" t="s">
         <v>248</v>
@@ -2083,7 +2080,7 @@
         <v>52</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -2103,7 +2100,7 @@
         <v>53</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -2123,7 +2120,7 @@
         <v>55</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -2143,7 +2140,7 @@
         <v>57</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -2163,7 +2160,7 @@
         <v>59</v>
       </c>
       <c r="F22" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -2183,7 +2180,7 @@
         <v>61</v>
       </c>
       <c r="F23" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -2203,7 +2200,7 @@
         <v>63</v>
       </c>
       <c r="F24" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -2223,7 +2220,7 @@
         <v>65</v>
       </c>
       <c r="F25" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -2275,7 +2272,7 @@
         <v>2</v>
       </c>
       <c r="I1" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="J1" t="s">
         <v>15</v>
@@ -2343,7 +2340,7 @@
         <v>13</v>
       </c>
       <c r="I3" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J3" t="s">
         <v>188</v>
@@ -2381,7 +2378,7 @@
         <v>180</v>
       </c>
       <c r="J4" t="s">
-        <v>189</v>
+        <v>52</v>
       </c>
       <c r="K4" t="s">
         <v>201</v>
@@ -2414,7 +2411,7 @@
         <v>13</v>
       </c>
       <c r="I5" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J5" t="s">
         <v>189</v>
@@ -2482,7 +2479,7 @@
         <v>13</v>
       </c>
       <c r="I7" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J7" t="s">
         <v>190</v>
@@ -2550,7 +2547,7 @@
         <v>13</v>
       </c>
       <c r="I9" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J9" t="s">
         <v>191</v>
@@ -2717,7 +2714,7 @@
         <v>13</v>
       </c>
       <c r="I14" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J14" t="s">
         <v>192</v>
@@ -2785,7 +2782,7 @@
         <v>13</v>
       </c>
       <c r="I16" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J16" t="s">
         <v>193</v>
@@ -2885,7 +2882,7 @@
         <v>13</v>
       </c>
       <c r="I19" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J19" t="s">
         <v>14</v>
@@ -3139,16 +3136,16 @@
         <v>75</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>316</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>318</v>
       </c>
       <c r="K1"/>
     </row>
@@ -3166,19 +3163,19 @@
         <v>77</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="F2" t="s">
         <v>116</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="I2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -3195,19 +3192,19 @@
         <v>79</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F3" t="s">
         <v>117</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="I3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -3215,25 +3212,25 @@
         <v>138</v>
       </c>
       <c r="B4" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F4" t="s">
         <v>118</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>198</v>
@@ -3253,22 +3250,22 @@
         <v>81</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F5" t="s">
         <v>119</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -3285,22 +3282,22 @@
         <v>83</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="F6" t="s">
         <v>120</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -3317,22 +3314,22 @@
         <v>85</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F7" t="s">
         <v>121</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -3349,19 +3346,19 @@
         <v>87</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F8" t="s">
         <v>122</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="I8" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -3378,22 +3375,22 @@
         <v>89</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F9" t="s">
         <v>123</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -3410,19 +3407,19 @@
         <v>91</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="F10" t="s">
         <v>124</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -3439,22 +3436,22 @@
         <v>93</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F11" t="s">
         <v>125</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -3471,22 +3468,22 @@
         <v>95</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F12" t="s">
         <v>126</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -3503,19 +3500,19 @@
         <v>97</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F13" t="s">
         <v>127</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -3529,25 +3526,25 @@
         <v>98</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F14" t="s">
         <v>128</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -3564,22 +3561,22 @@
         <v>100</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="F15" t="s">
         <v>129</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -3596,13 +3593,13 @@
         <v>102</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F16" t="s">
         <v>130</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -3619,22 +3616,22 @@
         <v>104</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="F17" t="s">
         <v>131</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -3651,22 +3648,22 @@
         <v>106</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="F18" t="s">
         <v>132</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -3674,7 +3671,7 @@
         <v>107</v>
       </c>
       <c r="B19" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C19" t="s">
         <v>107</v>
@@ -3683,13 +3680,13 @@
         <v>108</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F19" t="s">
         <v>133</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -3706,22 +3703,22 @@
         <v>33</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F20" t="s">
         <v>134</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -3738,22 +3735,22 @@
         <v>111</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F21" t="s">
         <v>135</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -3770,22 +3767,22 @@
         <v>113</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F22" t="s">
         <v>136</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -3802,22 +3799,22 @@
         <v>115</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F23" t="s">
         <v>137</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -3825,7 +3822,7 @@
         <v>208</v>
       </c>
       <c r="F26" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -3833,7 +3830,7 @@
         <v>209</v>
       </c>
       <c r="F27" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -3841,7 +3838,7 @@
         <v>210</v>
       </c>
       <c r="F28" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -3849,18 +3846,18 @@
         <v>211</v>
       </c>
       <c r="F29" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E30" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F30" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -3868,10 +3865,10 @@
         <v>213</v>
       </c>
       <c r="F31" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -3879,10 +3876,10 @@
         <v>214</v>
       </c>
       <c r="F32" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -3907,15 +3904,15 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B3">
         <v>9</v>
@@ -3923,7 +3920,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>290</v>
+        <v>402</v>
       </c>
       <c r="B4">
         <v>4</v>
@@ -3949,7 +3946,7 @@
         <v>256</v>
       </c>
       <c r="G6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -4035,7 +4032,7 @@
         <v>263</v>
       </c>
       <c r="B10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C10" t="s">
         <v>264</v>
@@ -4061,7 +4058,7 @@
         <v>266</v>
       </c>
       <c r="B11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C11" t="s">
         <v>266</v>
@@ -4084,16 +4081,16 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E12" t="s">
         <v>130</v>
@@ -4110,16 +4107,16 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>281</v>
+      </c>
+      <c r="B13" t="s">
         <v>282</v>
       </c>
-      <c r="B13" t="s">
-        <v>283</v>
-      </c>
       <c r="C13" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E13" t="s">
         <v>130</v>
@@ -4197,7 +4194,7 @@
         <v>273</v>
       </c>
       <c r="D16" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E16" t="s">
         <v>203</v>
@@ -4214,16 +4211,16 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>276</v>
+      </c>
+      <c r="B17" t="s">
+        <v>279</v>
+      </c>
+      <c r="C17" t="s">
+        <v>276</v>
+      </c>
+      <c r="D17" t="s">
         <v>274</v>
-      </c>
-      <c r="B17" t="s">
-        <v>280</v>
-      </c>
-      <c r="C17" t="s">
-        <v>277</v>
-      </c>
-      <c r="D17" t="s">
-        <v>275</v>
       </c>
       <c r="E17" t="s">
         <v>123</v>

</xml_diff>

<commit_message>
Fix errors in source Units_Prefixes.xls
Add english definition for second1960
Fix english candela 1979 definition so that 1/683 appears in math mode
</commit_message>
<xml_diff>
--- a/CUQ/_docs/Units_Prefixes.xlsx
+++ b/CUQ/_docs/Units_Prefixes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gruber04\git_repos\BIPM\Semantic-SI\CUQ\_docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\git_projects\SI-Reference-Point-2023\CUQ\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D097FE6C-DDE8-4D56-ADA6-6312EAC8C8CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFBFBA51-8A43-42A2-9585-ECF44E74CE29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-8310" windowWidth="38640" windowHeight="21390" activeTab="1" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
+    <workbookView xWindow="30555" yWindow="90" windowWidth="20940" windowHeight="14250" activeTab="1" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
   </bookViews>
   <sheets>
     <sheet name="Prefixes" sheetId="3" r:id="rId1"/>
@@ -47,9 +47,9 @@
   <commentList>
     <comment ref="F1" authorId="0" shapeId="0" xr:uid="{7938BEDB-7423-A84A-A317-D05AD2B442B6}">
       <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
     These will have ‘e’ and ‘f’ appended in code for language.</t>
       </text>
     </comment>
@@ -65,9 +65,9 @@
   <commentList>
     <comment ref="H1" authorId="0" shapeId="0" xr:uid="{5112C8FC-AB31-C04F-B4F8-A98CC949116C}">
       <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
     These will have ‘e’ and ‘f’ appended in code for language.</t>
       </text>
     </comment>
@@ -83,9 +83,9 @@
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0" xr:uid="{491B122B-80C3-6B46-8D7B-5F7258CFBC1C}">
       <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
     These will have ‘e’ and ‘f’ appended in code for language.</t>
       </text>
     </comment>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="404">
   <si>
     <t>hasStartValidity</t>
   </si>
@@ -676,9 +676,6 @@
   </si>
   <si>
     <t>AvogadroConstant</t>
-  </si>
-  <si>
-    <t>The candela is the luminous intensity, in a given direction, of a source that emits monochromatic radiation of frequency \(540 \times 10^{12}\) hertz and that has a radiant intensity in that direction of 1/683 watt per steradian.</t>
   </si>
   <si>
     <t>The kilogram is the unit of mass; it is equal to the mass of the international prototype of the kilogram.</t>
@@ -1376,6 +1373,12 @@
   </si>
   <si>
     <t>Le mètre est la longueur égale à @mvwv@ longueurs d'onde dans le vide de la radiation correspondant à la transition entre les niveaux @porb@ et @dorb@ de l'atome de krypton 86.</t>
+  </si>
+  <si>
+    <t>The second is the fraction @secf@ of the tropical year for 1900 January 0 at 12 hours ephemeris time.</t>
+  </si>
+  <si>
+    <t>The candela is the luminous intensity, in a given direction, of a source that emits monochromatic radiation of frequency \(540 \times 10^{12}\) hertz and that has a radiant intensity in that direction of @radi@ watt per steradian.</t>
   </si>
 </sst>
 </file>
@@ -1432,7 +1435,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1445,12 +1448,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1472,7 +1473,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1820,7 +1821,7 @@
         <v>2</v>
       </c>
       <c r="G1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1840,7 +1841,7 @@
         <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1860,7 +1861,7 @@
         <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1880,7 +1881,7 @@
         <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1888,10 +1889,10 @@
         <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D5" s="1">
         <v>1E+21</v>
@@ -1900,7 +1901,7 @@
         <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1920,7 +1921,7 @@
         <v>29</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1931,7 +1932,7 @@
         <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D7" s="1">
         <v>1000000000000000</v>
@@ -1940,7 +1941,7 @@
         <v>31</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1951,7 +1952,7 @@
         <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D8" s="1">
         <v>1000000000000</v>
@@ -1960,7 +1961,7 @@
         <v>33</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1980,7 +1981,7 @@
         <v>35</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1991,7 +1992,7 @@
         <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D10" s="1">
         <v>1000000</v>
@@ -2000,7 +2001,7 @@
         <v>37</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -2020,7 +2021,7 @@
         <v>39</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -2040,7 +2041,7 @@
         <v>41</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -2051,7 +2052,7 @@
         <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D13" s="1">
         <v>10</v>
@@ -2060,7 +2061,7 @@
         <v>43</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -2071,7 +2072,7 @@
         <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="D14" s="1">
         <v>0.1</v>
@@ -2080,7 +2081,7 @@
         <v>45</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -2100,7 +2101,7 @@
         <v>47</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -2120,7 +2121,7 @@
         <v>49</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2137,13 +2138,13 @@
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G17" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -2163,18 +2164,18 @@
         <v>52</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B19" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C19" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D19" s="1">
         <v>9.9999999999999998E-13</v>
@@ -2183,7 +2184,7 @@
         <v>53</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -2203,7 +2204,7 @@
         <v>55</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -2223,7 +2224,7 @@
         <v>57</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -2243,7 +2244,7 @@
         <v>59</v>
       </c>
       <c r="F22" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -2263,7 +2264,7 @@
         <v>61</v>
       </c>
       <c r="F23" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -2283,7 +2284,7 @@
         <v>63</v>
       </c>
       <c r="F24" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -2303,7 +2304,7 @@
         <v>65</v>
       </c>
       <c r="F25" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -2317,665 +2318,667 @@
   <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.375" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.375" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.125" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="79.375" style="10" customWidth="1"/>
-    <col min="7" max="7" width="42.375" style="10" customWidth="1"/>
-    <col min="8" max="8" width="19.625" style="10" customWidth="1"/>
-    <col min="9" max="9" width="102" style="10" customWidth="1"/>
-    <col min="10" max="10" width="29" style="10" customWidth="1"/>
-    <col min="11" max="16384" width="10.875" style="10"/>
+    <col min="1" max="1" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="79.375" customWidth="1"/>
+    <col min="7" max="7" width="42.375" customWidth="1"/>
+    <col min="8" max="8" width="19.625" customWidth="1"/>
+    <col min="9" max="9" width="102" customWidth="1"/>
+    <col min="10" max="10" width="29" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" t="s">
         <v>71</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" t="s">
         <v>72</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" t="s">
         <v>73</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="10" t="s">
-        <v>297</v>
-      </c>
-      <c r="J1" s="10" t="s">
+      <c r="I1" t="s">
+        <v>296</v>
+      </c>
+      <c r="J1" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="K1" t="s">
         <v>75</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="L1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" t="s">
+        <v>222</v>
+      </c>
+      <c r="G2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H2" t="s">
+        <v>179</v>
+      </c>
+      <c r="K2" t="s">
+        <v>199</v>
+      </c>
+      <c r="L2" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="E2" s="11" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" t="s">
+        <v>158</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="E3"/>
+      <c r="F3" t="s">
+        <v>220</v>
+      </c>
+      <c r="G3" t="s">
+        <v>240</v>
+      </c>
+      <c r="H3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" t="s">
+        <v>330</v>
+      </c>
+      <c r="J3" t="s">
+        <v>188</v>
+      </c>
+      <c r="K3" t="s">
+        <v>199</v>
+      </c>
+      <c r="L3" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F4" t="s">
         <v>223</v>
       </c>
-      <c r="G2" s="10" t="s">
-        <v>222</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="K2" s="10" t="s">
+      <c r="G4" t="s">
+        <v>403</v>
+      </c>
+      <c r="H4" t="s">
+        <v>180</v>
+      </c>
+      <c r="J4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K4" t="s">
         <v>200</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="L4" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B5" t="s">
+        <v>160</v>
+      </c>
+      <c r="C5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5"/>
+      <c r="F5" t="s">
+        <v>239</v>
+      </c>
+      <c r="G5" t="s">
+        <v>241</v>
+      </c>
+      <c r="H5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" t="s">
+        <v>310</v>
+      </c>
+      <c r="J5" t="s">
+        <v>189</v>
+      </c>
+      <c r="K5" t="s">
+        <v>200</v>
+      </c>
+      <c r="L5" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="D3" s="11" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>161</v>
+      </c>
+      <c r="B6" t="s">
+        <v>161</v>
+      </c>
+      <c r="C6" t="s">
+        <v>161</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F6" t="s">
+        <v>250</v>
+      </c>
+      <c r="G6" t="s">
+        <v>249</v>
+      </c>
+      <c r="H6" t="s">
+        <v>181</v>
+      </c>
+      <c r="K6" t="s">
+        <v>201</v>
+      </c>
+      <c r="L6" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" t="s">
+        <v>162</v>
+      </c>
+      <c r="C7" t="s">
+        <v>162</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>241</v>
-      </c>
-      <c r="H3" s="10" t="s">
+      <c r="E7"/>
+      <c r="F7" t="s">
+        <v>237</v>
+      </c>
+      <c r="G7" t="s">
+        <v>238</v>
+      </c>
+      <c r="H7" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I7" t="s">
+        <v>328</v>
+      </c>
+      <c r="J7" t="s">
+        <v>190</v>
+      </c>
+      <c r="K7" t="s">
+        <v>201</v>
+      </c>
+      <c r="L7" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B8" t="s">
+        <v>168</v>
+      </c>
+      <c r="C8" t="s">
+        <v>169</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" t="s">
+        <v>142</v>
+      </c>
+      <c r="G8" t="s">
+        <v>194</v>
+      </c>
+      <c r="H8" t="s">
+        <v>182</v>
+      </c>
+      <c r="K8" t="s">
+        <v>202</v>
+      </c>
+      <c r="L8" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>164</v>
+      </c>
+      <c r="B9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C9" t="s">
+        <v>164</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E9"/>
+      <c r="F9" t="s">
+        <v>236</v>
+      </c>
+      <c r="G9" t="s">
+        <v>235</v>
+      </c>
+      <c r="H9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" t="s">
         <v>331</v>
       </c>
-      <c r="J3" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="K3" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="L3" s="10" t="s">
+      <c r="J9" t="s">
+        <v>191</v>
+      </c>
+      <c r="K9" t="s">
+        <v>202</v>
+      </c>
+      <c r="L9" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B10" t="s">
+        <v>170</v>
+      </c>
+      <c r="C10" t="s">
+        <v>171</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="F10" t="s">
+        <v>398</v>
+      </c>
+      <c r="G10" t="s">
+        <v>195</v>
+      </c>
+      <c r="H10" t="s">
+        <v>183</v>
+      </c>
+      <c r="K10" t="s">
+        <v>203</v>
+      </c>
+      <c r="L10" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>173</v>
+      </c>
+      <c r="B11" t="s">
+        <v>172</v>
+      </c>
+      <c r="C11" t="s">
+        <v>173</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="F11" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="E4" s="11" t="s">
+      <c r="G11" t="s">
+        <v>224</v>
+      </c>
+      <c r="H11" t="s">
+        <v>184</v>
+      </c>
+      <c r="K11" t="s">
+        <v>203</v>
+      </c>
+      <c r="L11" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>175</v>
+      </c>
+      <c r="B12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C12" t="s">
+        <v>175</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>401</v>
+      </c>
+      <c r="G12" t="s">
+        <v>225</v>
+      </c>
+      <c r="H12" t="s">
+        <v>185</v>
+      </c>
+      <c r="K12" t="s">
+        <v>203</v>
+      </c>
+      <c r="L12" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>177</v>
+      </c>
+      <c r="B13" t="s">
+        <v>176</v>
+      </c>
+      <c r="C13" t="s">
+        <v>177</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>194</v>
-      </c>
-      <c r="H4" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="J4" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="L4" s="10" t="s">
+      <c r="F13" t="s">
+        <v>233</v>
+      </c>
+      <c r="G13" t="s">
+        <v>234</v>
+      </c>
+      <c r="H13" t="s">
+        <v>186</v>
+      </c>
+      <c r="J13" t="s">
+        <v>192</v>
+      </c>
+      <c r="K13" t="s">
+        <v>203</v>
+      </c>
+      <c r="L13" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>166</v>
+      </c>
+      <c r="B14" t="s">
+        <v>165</v>
+      </c>
+      <c r="C14" t="s">
+        <v>166</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14"/>
+      <c r="F14" t="s">
+        <v>232</v>
+      </c>
+      <c r="G14" t="s">
+        <v>226</v>
+      </c>
+      <c r="H14" t="s">
+        <v>13</v>
+      </c>
+      <c r="I14" t="s">
+        <v>332</v>
+      </c>
+      <c r="J14" t="s">
+        <v>192</v>
+      </c>
+      <c r="K14" t="s">
+        <v>203</v>
+      </c>
+      <c r="L14" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="D5" s="11" t="s">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>178</v>
+      </c>
+      <c r="B15" t="s">
+        <v>178</v>
+      </c>
+      <c r="C15" t="s">
+        <v>178</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F15" t="s">
+        <v>145</v>
+      </c>
+      <c r="G15" t="s">
+        <v>196</v>
+      </c>
+      <c r="H15" t="s">
+        <v>187</v>
+      </c>
+      <c r="K15" t="s">
+        <v>204</v>
+      </c>
+      <c r="L15" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>167</v>
+      </c>
+      <c r="B16" t="s">
+        <v>167</v>
+      </c>
+      <c r="C16" t="s">
+        <v>167</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>242</v>
-      </c>
-      <c r="H5" s="10" t="s">
+      <c r="E16"/>
+      <c r="F16" t="s">
+        <v>399</v>
+      </c>
+      <c r="G16" t="s">
+        <v>227</v>
+      </c>
+      <c r="H16" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="10" t="s">
-        <v>311</v>
-      </c>
-      <c r="J5" s="10" t="s">
-        <v>189</v>
-      </c>
-      <c r="K5" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="L5" s="10" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="D6" s="11" t="s">
+      <c r="I16" t="s">
+        <v>329</v>
+      </c>
+      <c r="J16" t="s">
+        <v>193</v>
+      </c>
+      <c r="K16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L16" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="F17" t="s">
+        <v>400</v>
+      </c>
+      <c r="G17" t="s">
+        <v>402</v>
+      </c>
+      <c r="H17" t="s">
+        <v>6</v>
+      </c>
+      <c r="K17" t="s">
+        <v>205</v>
+      </c>
+      <c r="L17" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E18" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>251</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="K6" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="L6" s="10" t="s">
+      <c r="F18" t="s">
+        <v>231</v>
+      </c>
+      <c r="G18" t="s">
+        <v>228</v>
+      </c>
+      <c r="H18" t="s">
+        <v>10</v>
+      </c>
+      <c r="J18" t="s">
+        <v>14</v>
+      </c>
+      <c r="K18" t="s">
+        <v>205</v>
+      </c>
+      <c r="L18" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19"/>
+      <c r="F19" t="s">
+        <v>230</v>
+      </c>
+      <c r="G19" t="s">
+        <v>229</v>
+      </c>
+      <c r="H19" t="s">
+        <v>13</v>
+      </c>
+      <c r="I19" t="s">
+        <v>333</v>
+      </c>
+      <c r="J19" t="s">
+        <v>14</v>
+      </c>
+      <c r="K19" t="s">
+        <v>205</v>
+      </c>
+      <c r="L19" t="s">
         <v>247</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>329</v>
-      </c>
-      <c r="J7" s="10" t="s">
-        <v>190</v>
-      </c>
-      <c r="K7" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="L7" s="10" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>182</v>
-      </c>
-      <c r="K8" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="L8" s="10" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>332</v>
-      </c>
-      <c r="J9" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="L9" s="10" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>399</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>183</v>
-      </c>
-      <c r="K10" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="L10" s="10" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>249</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="K11" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="L11" s="10" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>402</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>226</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="K12" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="L12" s="10" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>177</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="J13" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="K13" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="L13" s="10" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I14" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="J14" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="K14" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="L14" s="10" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="K15" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="L15" s="10" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10" t="s">
-        <v>400</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>330</v>
-      </c>
-      <c r="J16" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="K16" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="L16" s="10" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>199</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>401</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="K17" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="L17" s="10" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>232</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="J18" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="K18" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="L18" s="10" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I19" s="10" t="s">
-        <v>334</v>
-      </c>
-      <c r="J19" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="K19" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="L19" s="10" t="s">
-        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -3000,7 +3003,7 @@
         <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E1" t="s">
         <v>16</v>
@@ -3008,16 +3011,16 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E2" t="s">
         <v>139</v>
@@ -3031,16 +3034,16 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E3" t="s">
         <v>140</v>
@@ -3054,19 +3057,19 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F4" t="s">
         <v>161</v>
@@ -3077,16 +3080,16 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E5" t="s">
         <v>141</v>
@@ -3100,16 +3103,16 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E6" t="s">
         <v>49</v>
@@ -3132,16 +3135,16 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E7" t="s">
         <v>144</v>
@@ -3155,16 +3158,16 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
@@ -3220,16 +3223,16 @@
         <v>75</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="K1"/>
     </row>
@@ -3247,19 +3250,19 @@
         <v>77</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F2" t="s">
         <v>116</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="I2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -3276,19 +3279,19 @@
         <v>79</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F3" t="s">
         <v>117</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="I3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -3296,28 +3299,28 @@
         <v>138</v>
       </c>
       <c r="B4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F4" t="s">
         <v>118</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -3334,22 +3337,22 @@
         <v>81</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F5" t="s">
         <v>119</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>370</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -3366,22 +3369,22 @@
         <v>83</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F6" t="s">
         <v>120</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -3398,22 +3401,22 @@
         <v>85</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F7" t="s">
         <v>121</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -3430,19 +3433,19 @@
         <v>87</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F8" t="s">
         <v>122</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="I8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -3459,22 +3462,22 @@
         <v>89</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F9" t="s">
         <v>123</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -3491,19 +3494,19 @@
         <v>91</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F10" t="s">
         <v>124</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -3520,22 +3523,22 @@
         <v>93</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F11" t="s">
         <v>125</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -3552,22 +3555,22 @@
         <v>95</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F12" t="s">
         <v>126</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -3584,19 +3587,19 @@
         <v>97</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F13" t="s">
         <v>127</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -3610,25 +3613,25 @@
         <v>98</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F14" t="s">
         <v>128</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -3645,22 +3648,22 @@
         <v>100</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F15" t="s">
         <v>129</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -3677,13 +3680,13 @@
         <v>102</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F16" t="s">
         <v>130</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -3700,22 +3703,22 @@
         <v>104</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F17" t="s">
         <v>131</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -3732,22 +3735,22 @@
         <v>106</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F18" t="s">
         <v>132</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -3755,7 +3758,7 @@
         <v>107</v>
       </c>
       <c r="B19" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C19" t="s">
         <v>107</v>
@@ -3764,13 +3767,13 @@
         <v>108</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F19" t="s">
         <v>133</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -3787,22 +3790,22 @@
         <v>33</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F20" t="s">
         <v>134</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -3819,22 +3822,22 @@
         <v>111</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F21" t="s">
         <v>135</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -3851,22 +3854,22 @@
         <v>113</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F22" t="s">
         <v>136</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -3883,87 +3886,87 @@
         <v>115</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F23" t="s">
         <v>137</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E26" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F26" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E27" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F27" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E28" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F28" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E29" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F29" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E30" s="8" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F30" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E31" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F31" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E32" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F32" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -3988,15 +3991,15 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B3">
         <v>9</v>
@@ -4004,7 +4007,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B4">
         <v>4</v>
@@ -4027,33 +4030,33 @@
         <v>75</v>
       </c>
       <c r="F6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>252</v>
+      </c>
+      <c r="B7" t="s">
+        <v>252</v>
+      </c>
+      <c r="C7" t="s">
+        <v>252</v>
+      </c>
+      <c r="D7" t="s">
         <v>253</v>
       </c>
-      <c r="B7" t="s">
-        <v>253</v>
-      </c>
-      <c r="C7" t="s">
-        <v>253</v>
-      </c>
-      <c r="D7" t="s">
-        <v>254</v>
-      </c>
       <c r="E7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F7">
         <v>60</v>
       </c>
       <c r="G7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -4061,25 +4064,25 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D8" t="s">
         <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F8">
         <v>3600</v>
       </c>
       <c r="G8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -4087,25 +4090,25 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D9" t="s">
         <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F9">
         <v>86400</v>
       </c>
       <c r="G9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -4113,25 +4116,25 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>258</v>
+      </c>
+      <c r="B10" t="s">
+        <v>272</v>
+      </c>
+      <c r="C10" t="s">
         <v>259</v>
       </c>
-      <c r="B10" t="s">
-        <v>273</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>260</v>
       </c>
-      <c r="D10" t="s">
-        <v>261</v>
-      </c>
       <c r="E10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F10" s="7">
         <v>149597870700</v>
       </c>
       <c r="G10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -4139,16 +4142,16 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>261</v>
+      </c>
+      <c r="B11" t="s">
+        <v>273</v>
+      </c>
+      <c r="C11" t="s">
+        <v>261</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>262</v>
-      </c>
-      <c r="B11" t="s">
-        <v>274</v>
-      </c>
-      <c r="C11" t="s">
-        <v>262</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>263</v>
       </c>
       <c r="E11" t="s">
         <v>130</v>
@@ -4165,16 +4168,16 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E12" t="s">
         <v>130</v>
@@ -4191,16 +4194,16 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>276</v>
+      </c>
+      <c r="B13" t="s">
         <v>277</v>
       </c>
-      <c r="B13" t="s">
-        <v>278</v>
-      </c>
       <c r="C13" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E13" t="s">
         <v>130</v>
@@ -4217,25 +4220,25 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>263</v>
+      </c>
+      <c r="B14" t="s">
+        <v>263</v>
+      </c>
+      <c r="C14" t="s">
+        <v>263</v>
+      </c>
+      <c r="D14" t="s">
         <v>264</v>
       </c>
-      <c r="B14" t="s">
-        <v>264</v>
-      </c>
-      <c r="C14" t="s">
-        <v>264</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>265</v>
-      </c>
-      <c r="E14" t="s">
-        <v>266</v>
       </c>
       <c r="F14">
         <v>1E-3</v>
       </c>
       <c r="G14" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H14">
         <v>3</v>
@@ -4243,25 +4246,25 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>266</v>
+      </c>
+      <c r="B15" t="s">
+        <v>266</v>
+      </c>
+      <c r="C15" t="s">
+        <v>266</v>
+      </c>
+      <c r="D15" t="s">
         <v>267</v>
       </c>
-      <c r="B15" t="s">
-        <v>267</v>
-      </c>
-      <c r="C15" t="s">
-        <v>267</v>
-      </c>
-      <c r="D15" t="s">
-        <v>268</v>
-      </c>
       <c r="E15" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F15">
         <v>1000</v>
       </c>
       <c r="G15" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -4269,25 +4272,25 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B16" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C16" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D16" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E16" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F16" s="6">
         <v>1.6605390666E-27</v>
       </c>
       <c r="G16" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -4295,16 +4298,16 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B17" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C17" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D17" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E17" t="s">
         <v>123</v>

</xml_diff>

<commit_message>
Removed wls dep in units, still wip for latex format
</commit_message>
<xml_diff>
--- a/CUQ/_docs/Units_Prefixes.xlsx
+++ b/CUQ/_docs/Units_Prefixes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\git_projects\SI-Reference-Point-2023\CUQ\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFBFBA51-8A43-42A2-9585-ECF44E74CE29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D90FAEA-042E-4B75-8F99-8B1DB9EA3EF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30555" yWindow="90" windowWidth="20940" windowHeight="14250" activeTab="1" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
+    <workbookView xWindow="31725" yWindow="960" windowWidth="20940" windowHeight="14250" activeTab="4" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
   </bookViews>
   <sheets>
     <sheet name="Prefixes" sheetId="3" r:id="rId1"/>
@@ -315,9 +315,6 @@
     <t>hasDefiningText_fr</t>
   </si>
   <si>
-    <t>hasDefiingText_en</t>
-  </si>
-  <si>
     <t>Symbol</t>
   </si>
   <si>
@@ -849,9 +846,6 @@
     <t>Le kelvin, unité de température thermodynamique, est la fraction @celi@ de la température thermodynamique du point triple de l'eau.</t>
   </si>
   <si>
-    <t>conversionfactor</t>
-  </si>
-  <si>
     <t>minute</t>
   </si>
   <si>
@@ -934,9 +928,6 @@
   </si>
   <si>
     <t>@arcs@</t>
-  </si>
-  <si>
-    <t>conversionsiunit</t>
   </si>
   <si>
     <t>SI Brochure</t>
@@ -1379,6 +1370,15 @@
   </si>
   <si>
     <t>The candela is the luminous intensity, in a given direction, of a source that emits monochromatic radiation of frequency \(540 \times 10^{12}\) hertz and that has a radiant intensity in that direction of @radi@ watt per steradian.</t>
+  </si>
+  <si>
+    <t>hasDefiningText_en</t>
+  </si>
+  <si>
+    <t>ConversionFactor</t>
+  </si>
+  <si>
+    <t>ConversionUnit</t>
   </si>
 </sst>
 </file>
@@ -1821,7 +1821,7 @@
         <v>2</v>
       </c>
       <c r="G1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1841,7 +1841,7 @@
         <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1861,7 +1861,7 @@
         <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1881,7 +1881,7 @@
         <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1889,10 +1889,10 @@
         <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D5" s="1">
         <v>1E+21</v>
@@ -1901,7 +1901,7 @@
         <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1921,7 +1921,7 @@
         <v>29</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1932,7 +1932,7 @@
         <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="D7" s="1">
         <v>1000000000000000</v>
@@ -1941,7 +1941,7 @@
         <v>31</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1952,7 +1952,7 @@
         <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="D8" s="1">
         <v>1000000000000</v>
@@ -1961,7 +1961,7 @@
         <v>33</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1981,7 +1981,7 @@
         <v>35</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1992,7 +1992,7 @@
         <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="D10" s="1">
         <v>1000000</v>
@@ -2001,7 +2001,7 @@
         <v>37</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -2021,7 +2021,7 @@
         <v>39</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -2041,7 +2041,7 @@
         <v>41</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -2052,7 +2052,7 @@
         <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="D13" s="1">
         <v>10</v>
@@ -2061,7 +2061,7 @@
         <v>43</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -2072,7 +2072,7 @@
         <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="D14" s="1">
         <v>0.1</v>
@@ -2081,7 +2081,7 @@
         <v>45</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -2101,7 +2101,7 @@
         <v>47</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -2121,7 +2121,7 @@
         <v>49</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -2138,13 +2138,13 @@
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="G17" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -2164,18 +2164,18 @@
         <v>52</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D19" s="1">
         <v>9.9999999999999998E-13</v>
@@ -2184,7 +2184,7 @@
         <v>53</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -2204,7 +2204,7 @@
         <v>55</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -2224,7 +2224,7 @@
         <v>57</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -2244,7 +2244,7 @@
         <v>59</v>
       </c>
       <c r="F22" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -2264,7 +2264,7 @@
         <v>61</v>
       </c>
       <c r="F23" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -2284,7 +2284,7 @@
         <v>63</v>
       </c>
       <c r="F24" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -2304,7 +2304,7 @@
         <v>65</v>
       </c>
       <c r="F25" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -2350,172 +2350,172 @@
         <v>72</v>
       </c>
       <c r="G1" t="s">
-        <v>73</v>
+        <v>401</v>
       </c>
       <c r="H1" t="s">
         <v>2</v>
       </c>
       <c r="I1" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="J1" t="s">
         <v>15</v>
       </c>
       <c r="K1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C2" t="s">
         <v>155</v>
       </c>
-      <c r="C2" t="s">
-        <v>156</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>68</v>
       </c>
       <c r="F2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="L2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C3" t="s">
         <v>157</v>
-      </c>
-      <c r="C3" t="s">
-        <v>158</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>68</v>
       </c>
       <c r="E3"/>
       <c r="F3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H3" t="s">
         <v>13</v>
       </c>
       <c r="I3" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="J3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="L3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="F4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G4" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="H4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J4" t="s">
         <v>52</v>
       </c>
       <c r="K4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="L4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>68</v>
       </c>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H5" t="s">
         <v>13</v>
       </c>
       <c r="I5" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="J5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="L5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>67</v>
@@ -2524,358 +2524,358 @@
         <v>69</v>
       </c>
       <c r="F6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="L6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>68</v>
       </c>
       <c r="E7"/>
       <c r="F7" t="s">
+        <v>236</v>
+      </c>
+      <c r="G7" t="s">
         <v>237</v>
-      </c>
-      <c r="G7" t="s">
-        <v>238</v>
       </c>
       <c r="H7" t="s">
         <v>13</v>
       </c>
       <c r="I7" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="J7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="K7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="L7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B8" t="s">
+        <v>167</v>
+      </c>
+      <c r="C8" t="s">
         <v>168</v>
       </c>
-      <c r="C8" t="s">
-        <v>169</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>69</v>
       </c>
       <c r="F8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="L8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C9" t="s">
         <v>163</v>
-      </c>
-      <c r="C9" t="s">
-        <v>164</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>68</v>
       </c>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H9" t="s">
         <v>13</v>
       </c>
       <c r="I9" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="J9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="K9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="L9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B10" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" t="s">
         <v>170</v>
       </c>
-      <c r="C10" t="s">
-        <v>171</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F10" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="G10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C11" t="s">
         <v>172</v>
       </c>
-      <c r="C11" t="s">
-        <v>173</v>
-      </c>
       <c r="D11" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="F11" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="K11" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B12" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" t="s">
         <v>174</v>
-      </c>
-      <c r="C12" t="s">
-        <v>175</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>66</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="G12" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K12" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L12" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B13" t="s">
+        <v>175</v>
+      </c>
+      <c r="C13" t="s">
         <v>176</v>
       </c>
-      <c r="C13" t="s">
-        <v>177</v>
-      </c>
       <c r="D13" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>69</v>
       </c>
       <c r="F13" t="s">
+        <v>232</v>
+      </c>
+      <c r="G13" t="s">
         <v>233</v>
       </c>
-      <c r="G13" t="s">
-        <v>234</v>
-      </c>
       <c r="H13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="K13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C14" t="s">
         <v>165</v>
-      </c>
-      <c r="C14" t="s">
-        <v>166</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>68</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H14" t="s">
         <v>13</v>
       </c>
       <c r="I14" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="J14" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="K14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>69</v>
       </c>
       <c r="F15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L15" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>68</v>
       </c>
       <c r="E16"/>
       <c r="F16" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="G16" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H16" t="s">
         <v>13</v>
       </c>
       <c r="I16" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="J16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L16" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -2892,22 +2892,22 @@
         <v>66</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F17" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="G17" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="H17" t="s">
         <v>6</v>
       </c>
       <c r="K17" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L17" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -2927,10 +2927,10 @@
         <v>69</v>
       </c>
       <c r="F18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G18" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H18" t="s">
         <v>10</v>
@@ -2939,10 +2939,10 @@
         <v>14</v>
       </c>
       <c r="K18" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L18" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
@@ -2960,25 +2960,25 @@
       </c>
       <c r="E19"/>
       <c r="F19" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G19" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H19" t="s">
         <v>13</v>
       </c>
       <c r="I19" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="J19" t="s">
         <v>14</v>
       </c>
       <c r="K19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L19" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -3003,7 +3003,7 @@
         <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E1" t="s">
         <v>16</v>
@@ -3011,163 +3011,163 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G3" t="s">
         <v>159</v>
-      </c>
-      <c r="G3" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G4" t="s">
         <v>161</v>
-      </c>
-      <c r="G4" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E6" t="s">
         <v>49</v>
       </c>
       <c r="F6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
@@ -3214,759 +3214,759 @@
         <v>71</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>308</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>311</v>
       </c>
       <c r="K1"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="F2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="I2" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="I3" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B4" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C4" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>83</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="F6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B7" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" t="s">
-        <v>84</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C8" t="s">
-        <v>86</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="E8" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="I8" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B10" t="s">
-        <v>90</v>
-      </c>
-      <c r="C10" t="s">
-        <v>90</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="E10" s="2" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" t="s">
+        <v>91</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B11" t="s">
-        <v>92</v>
-      </c>
-      <c r="C11" t="s">
-        <v>92</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>93</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" t="s">
-        <v>94</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>95</v>
-      </c>
       <c r="E12" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>95</v>
+      </c>
+      <c r="B13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B13" t="s">
-        <v>96</v>
-      </c>
-      <c r="C13" t="s">
-        <v>96</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" t="s">
+        <v>98</v>
+      </c>
+      <c r="C15" t="s">
+        <v>98</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B15" t="s">
-        <v>99</v>
-      </c>
-      <c r="C15" t="s">
-        <v>99</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>100</v>
-      </c>
       <c r="E15" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B16" t="s">
-        <v>101</v>
-      </c>
-      <c r="C16" t="s">
-        <v>101</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>102</v>
-      </c>
       <c r="E16" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" t="s">
+        <v>102</v>
+      </c>
+      <c r="C17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B17" t="s">
-        <v>103</v>
-      </c>
-      <c r="C17" t="s">
-        <v>103</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="E17" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B18" t="s">
-        <v>105</v>
-      </c>
-      <c r="C18" t="s">
-        <v>105</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="E18" s="2" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" t="s">
+        <v>393</v>
+      </c>
+      <c r="C19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B19" t="s">
-        <v>396</v>
-      </c>
-      <c r="C19" t="s">
-        <v>107</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="E19" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F19" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F20" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" t="s">
+        <v>109</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B21" t="s">
-        <v>110</v>
-      </c>
-      <c r="C21" t="s">
-        <v>110</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E21" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F21" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>111</v>
+      </c>
+      <c r="B22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C22" t="s">
-        <v>112</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>113</v>
-      </c>
       <c r="E22" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F22" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>113</v>
+      </c>
+      <c r="B23" t="s">
+        <v>113</v>
+      </c>
+      <c r="C23" t="s">
+        <v>113</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B23" t="s">
-        <v>114</v>
-      </c>
-      <c r="C23" t="s">
-        <v>114</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>115</v>
-      </c>
       <c r="E23" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F23" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E26" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F26" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E27" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F27" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E28" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F28" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E29" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F29" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E30" s="8" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F30" t="s">
+        <v>338</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>341</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E31" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F31" t="s">
+        <v>339</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>342</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E32" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F32" t="s">
+        <v>340</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>343</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -3991,15 +3991,15 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B2" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B3">
         <v>9</v>
@@ -4007,7 +4007,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="B4">
         <v>4</v>
@@ -4024,39 +4024,39 @@
         <v>71</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" t="s">
         <v>74</v>
       </c>
-      <c r="E6" t="s">
-        <v>75</v>
-      </c>
       <c r="F6" t="s">
-        <v>251</v>
+        <v>402</v>
       </c>
       <c r="G6" t="s">
-        <v>280</v>
+        <v>403</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="D7" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="E7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F7">
         <v>60</v>
       </c>
       <c r="G7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -4064,25 +4064,25 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B8" t="s">
+        <v>252</v>
+      </c>
+      <c r="C8" t="s">
         <v>254</v>
-      </c>
-      <c r="C8" t="s">
-        <v>256</v>
       </c>
       <c r="D8" t="s">
         <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F8">
         <v>3600</v>
       </c>
       <c r="G8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -4090,25 +4090,25 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B9" t="s">
+        <v>253</v>
+      </c>
+      <c r="C9" t="s">
         <v>255</v>
-      </c>
-      <c r="C9" t="s">
-        <v>257</v>
       </c>
       <c r="D9" t="s">
         <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F9">
         <v>86400</v>
       </c>
       <c r="G9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -4116,25 +4116,25 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>256</v>
+      </c>
+      <c r="B10" t="s">
+        <v>270</v>
+      </c>
+      <c r="C10" t="s">
+        <v>257</v>
+      </c>
+      <c r="D10" t="s">
         <v>258</v>
       </c>
-      <c r="B10" t="s">
-        <v>272</v>
-      </c>
-      <c r="C10" t="s">
-        <v>259</v>
-      </c>
-      <c r="D10" t="s">
-        <v>260</v>
-      </c>
       <c r="E10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F10" s="7">
         <v>149597870700</v>
       </c>
       <c r="G10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -4142,25 +4142,25 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B11" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C11" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F11" s="5">
         <v>1.7453292519943299E-2</v>
       </c>
       <c r="G11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -4168,25 +4168,25 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B12" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C12" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F12" s="5">
         <v>2.9088820866572201E-4</v>
       </c>
       <c r="G12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -4194,25 +4194,25 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B13" t="s">
+        <v>275</v>
+      </c>
+      <c r="C13" t="s">
+        <v>274</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C13" t="s">
-        <v>276</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>279</v>
-      </c>
       <c r="E13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F13" s="5">
         <v>4.8481368110953598E-6</v>
       </c>
       <c r="G13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H13">
         <v>1</v>
@@ -4220,25 +4220,25 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>261</v>
+      </c>
+      <c r="B14" t="s">
+        <v>261</v>
+      </c>
+      <c r="C14" t="s">
+        <v>261</v>
+      </c>
+      <c r="D14" t="s">
+        <v>262</v>
+      </c>
+      <c r="E14" t="s">
         <v>263</v>
-      </c>
-      <c r="B14" t="s">
-        <v>263</v>
-      </c>
-      <c r="C14" t="s">
-        <v>263</v>
-      </c>
-      <c r="D14" t="s">
-        <v>264</v>
-      </c>
-      <c r="E14" t="s">
-        <v>265</v>
       </c>
       <c r="F14">
         <v>1E-3</v>
       </c>
       <c r="G14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H14">
         <v>3</v>
@@ -4246,25 +4246,25 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B15" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C15" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D15" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E15" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F15">
         <v>1000</v>
       </c>
       <c r="G15" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -4272,25 +4272,25 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>266</v>
+      </c>
+      <c r="B16" t="s">
+        <v>266</v>
+      </c>
+      <c r="C16" t="s">
+        <v>266</v>
+      </c>
+      <c r="D16" t="s">
         <v>268</v>
       </c>
-      <c r="B16" t="s">
-        <v>268</v>
-      </c>
-      <c r="C16" t="s">
-        <v>268</v>
-      </c>
-      <c r="D16" t="s">
-        <v>270</v>
-      </c>
       <c r="E16" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F16" s="6">
         <v>1.6605390666E-27</v>
       </c>
       <c r="G16" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -4298,25 +4298,25 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B17" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C17" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D17" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F17" s="7">
         <v>1.6021766339999999E-19</v>
       </c>
       <c r="G17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H17">
         <v>1</v>

</xml_diff>

<commit_message>
SI-Reference-Point-2023-14 Addition of other JSON-LD outputs (via content negotiation) for other ...
Adding JSON-LD output for prefixes.  Updated the Units_Prefixes.xlsx file with datatypes for each scaling factor and added them to the Prefixes_ABox.py code.

command line 'curl http://127.0.0.1:8000/si-prefixes/ -H "Accept: application/ld+json" -o 'prefixes.jsonld''
</commit_message>
<xml_diff>
--- a/CUQ/_docs/Units_Prefixes.xlsx
+++ b/CUQ/_docs/Units_Prefixes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\fmeynadier\git_projects\SI-Reference-Point-2023\CUQ\_docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n00002621/PycharmProjects/SI-Reference-Point-2023/CUQ/_docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4004A2-C191-4509-828F-7CA95D7F9C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48BDB282-E8DB-F44E-9854-396DE8AF6A83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4215" yWindow="1920" windowWidth="23325" windowHeight="11295" activeTab="1" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
   </bookViews>
   <sheets>
     <sheet name="Prefixes" sheetId="3" r:id="rId1"/>
@@ -47,9 +47,9 @@
   <commentList>
     <comment ref="F1" authorId="0" shapeId="0" xr:uid="{7938BEDB-7423-A84A-A317-D05AD2B442B6}">
       <text>
-        <t>[Commentaire à thread]
-Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
-Commentaire :
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     These will have ‘e’ and ‘f’ appended in code for language.</t>
       </text>
     </comment>
@@ -65,9 +65,9 @@
   <commentList>
     <comment ref="H1" authorId="0" shapeId="0" xr:uid="{5112C8FC-AB31-C04F-B4F8-A98CC949116C}">
       <text>
-        <t>[Commentaire à thread]
-Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
-Commentaire :
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     These will have ‘e’ and ‘f’ appended in code for language.</t>
       </text>
     </comment>
@@ -83,9 +83,9 @@
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0" xr:uid="{491B122B-80C3-6B46-8D7B-5F7258CFBC1C}">
       <text>
-        <t>[Commentaire à thread]
-Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
-Commentaire :
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     These will have ‘e’ and ‘f’ appended in code for language.</t>
       </text>
     </comment>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="408">
   <si>
     <t>hasStartValidity</t>
   </si>
@@ -1379,6 +1379,18 @@
   </si>
   <si>
     <t>The candela is the luminous intensity, in a given direction, of a source that emits monochromatic radiation of frequency \(540 \times 10^{12}\) hertz and that has a radiant intensity in that direction of @radi@ watt per steradian.</t>
+  </si>
+  <si>
+    <t>datatype</t>
+  </si>
+  <si>
+    <t>integer</t>
+  </si>
+  <si>
+    <t>decimal</t>
+  </si>
+  <si>
+    <t>float</t>
   </si>
 </sst>
 </file>
@@ -1473,7 +1485,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1793,15 +1805,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A359D5A-52A8-E54D-810F-2890E8F81F39}">
-  <dimension ref="A1:G25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="10.875" style="2"/>
-    <col min="5" max="5" width="10.875" style="2"/>
-    <col min="6" max="6" width="20.875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" style="2"/>
+    <col min="5" max="5" width="10.83203125" style="2"/>
+    <col min="6" max="7" width="20.83203125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -1821,10 +1833,13 @@
         <v>2</v>
       </c>
       <c r="G1" t="s">
+        <v>404</v>
+      </c>
+      <c r="H1" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -1843,8 +1858,11 @@
       <c r="F2" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1863,8 +1881,11 @@
       <c r="F3" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -1883,8 +1904,11 @@
       <c r="F4" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -1903,8 +1927,11 @@
       <c r="F5" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -1923,8 +1950,11 @@
       <c r="F6" s="2" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -1943,8 +1973,11 @@
       <c r="F7" s="2" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1963,8 +1996,11 @@
       <c r="F8" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -1983,8 +2019,11 @@
       <c r="F9" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G9" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -2003,8 +2042,11 @@
       <c r="F10" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -2023,8 +2065,11 @@
       <c r="F11" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -2043,8 +2088,11 @@
       <c r="F12" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G12" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -2063,8 +2111,11 @@
       <c r="F13" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G13" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>44</v>
       </c>
@@ -2083,8 +2134,11 @@
       <c r="F14" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G14" s="2" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -2103,8 +2157,11 @@
       <c r="F15" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G15" s="2" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -2123,8 +2180,11 @@
       <c r="F16" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G16" s="2" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>50</v>
       </c>
@@ -2143,11 +2203,14 @@
       <c r="F17" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="H17" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>51</v>
       </c>
@@ -2166,8 +2229,11 @@
       <c r="F18" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G18" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>206</v>
       </c>
@@ -2186,8 +2252,11 @@
       <c r="F19" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G19" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -2206,8 +2275,11 @@
       <c r="F20" s="2" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G20" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>56</v>
       </c>
@@ -2226,8 +2298,11 @@
       <c r="F21" s="2" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G21" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>58</v>
       </c>
@@ -2246,8 +2321,11 @@
       <c r="F22" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G22" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>60</v>
       </c>
@@ -2266,8 +2344,11 @@
       <c r="F23" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G23" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -2286,8 +2367,11 @@
       <c r="F24" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G24" s="2" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -2305,6 +2389,9 @@
       </c>
       <c r="F25" t="s">
         <v>286</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>407</v>
       </c>
     </row>
   </sheetData>
@@ -2316,21 +2403,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DE8A68B-8B60-3949-B0A8-4A96CE4D68DA}">
   <dimension ref="A1:L19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="79.375" customWidth="1"/>
-    <col min="7" max="7" width="42.375" customWidth="1"/>
-    <col min="8" max="8" width="19.625" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="79.33203125" customWidth="1"/>
+    <col min="7" max="7" width="42.33203125" customWidth="1"/>
+    <col min="8" max="8" width="19.6640625" customWidth="1"/>
     <col min="9" max="9" width="102" customWidth="1"/>
     <col min="10" max="10" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -2368,7 +2455,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>156</v>
       </c>
@@ -2400,7 +2487,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>158</v>
       </c>
@@ -2436,7 +2523,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>159</v>
       </c>
@@ -2461,9 +2548,6 @@
       <c r="H4" t="s">
         <v>180</v>
       </c>
-      <c r="J4" t="s">
-        <v>189</v>
-      </c>
       <c r="K4" t="s">
         <v>200</v>
       </c>
@@ -2471,7 +2555,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>160</v>
       </c>
@@ -2507,7 +2591,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>161</v>
       </c>
@@ -2539,7 +2623,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>162</v>
       </c>
@@ -2575,7 +2659,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>169</v>
       </c>
@@ -2607,7 +2691,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>164</v>
       </c>
@@ -2643,7 +2727,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>171</v>
       </c>
@@ -2675,7 +2759,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>173</v>
       </c>
@@ -2707,7 +2791,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>175</v>
       </c>
@@ -2739,7 +2823,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>177</v>
       </c>
@@ -2774,7 +2858,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>166</v>
       </c>
@@ -2810,7 +2894,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>178</v>
       </c>
@@ -2842,7 +2926,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>167</v>
       </c>
@@ -2878,7 +2962,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -2910,7 +2994,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>7</v>
       </c>
@@ -2945,7 +3029,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -2990,9 +3074,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EF3A1C2-6A3C-474E-908C-FA60BE09F193}">
   <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -3009,7 +3093,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>207</v>
       </c>
@@ -3032,7 +3116,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>208</v>
       </c>
@@ -3055,7 +3139,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>209</v>
       </c>
@@ -3078,7 +3162,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>210</v>
       </c>
@@ -3101,7 +3185,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>211</v>
       </c>
@@ -3133,7 +3217,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>212</v>
       </c>
@@ -3156,7 +3240,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>213</v>
       </c>
@@ -3190,20 +3274,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{837449F3-3B63-3745-8303-091E9EC09344}">
   <dimension ref="A1:K32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.875" style="2"/>
-    <col min="5" max="5" width="21.125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="13.125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" style="2"/>
+    <col min="5" max="5" width="21.1640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="13.1640625" customWidth="1"/>
     <col min="7" max="7" width="26.5" style="2" customWidth="1"/>
-    <col min="8" max="8" width="47.875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="47.83203125" style="2" customWidth="1"/>
     <col min="9" max="9" width="189.5" style="2" customWidth="1"/>
     <col min="10" max="10" width="20" style="2" customWidth="1"/>
     <col min="11" max="11" width="21" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -3236,7 +3320,7 @@
       </c>
       <c r="K1"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>76</v>
       </c>
@@ -3265,7 +3349,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>78</v>
       </c>
@@ -3294,7 +3378,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>138</v>
       </c>
@@ -3323,7 +3407,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>80</v>
       </c>
@@ -3355,7 +3439,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>82</v>
       </c>
@@ -3387,7 +3471,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>84</v>
       </c>
@@ -3419,7 +3503,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>86</v>
       </c>
@@ -3448,7 +3532,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>88</v>
       </c>
@@ -3480,7 +3564,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>90</v>
       </c>
@@ -3509,7 +3593,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>92</v>
       </c>
@@ -3541,7 +3625,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>94</v>
       </c>
@@ -3573,7 +3657,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -3602,7 +3686,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>98</v>
       </c>
@@ -3634,7 +3718,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>99</v>
       </c>
@@ -3666,7 +3750,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>101</v>
       </c>
@@ -3689,7 +3773,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>103</v>
       </c>
@@ -3721,7 +3805,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>105</v>
       </c>
@@ -3753,7 +3837,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>107</v>
       </c>
@@ -3776,7 +3860,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>109</v>
       </c>
@@ -3808,7 +3892,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>110</v>
       </c>
@@ -3840,7 +3924,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>112</v>
       </c>
@@ -3872,7 +3956,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>114</v>
       </c>
@@ -3904,7 +3988,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E26" s="8" t="s">
         <v>207</v>
       </c>
@@ -3912,7 +3996,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E27" s="8" t="s">
         <v>208</v>
       </c>
@@ -3920,7 +4004,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E28" s="8" t="s">
         <v>209</v>
       </c>
@@ -3928,7 +4012,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E29" s="8" t="s">
         <v>210</v>
       </c>
@@ -3936,7 +4020,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E30" s="8" t="s">
         <v>334</v>
       </c>
@@ -3947,7 +4031,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E31" s="8" t="s">
         <v>212</v>
       </c>
@@ -3958,7 +4042,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E32" s="8" t="s">
         <v>213</v>
       </c>
@@ -3978,18 +4062,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC3BD8C3-F79C-5947-ABF9-F73A9D2E6571}">
   <dimension ref="A2:K27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.875" customWidth="1"/>
-    <col min="2" max="2" width="12.875" customWidth="1"/>
-    <col min="3" max="3" width="12.625" customWidth="1"/>
-    <col min="4" max="5" width="14.125" customWidth="1"/>
-    <col min="6" max="6" width="20.375" customWidth="1"/>
-    <col min="10" max="10" width="25.875" customWidth="1"/>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" customWidth="1"/>
+    <col min="4" max="5" width="14.1640625" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
+    <col min="10" max="10" width="25.83203125" customWidth="1"/>
     <col min="11" max="11" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>282</v>
       </c>
@@ -3997,7 +4081,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>283</v>
       </c>
@@ -4005,7 +4089,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>397</v>
       </c>
@@ -4013,7 +4097,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -4036,7 +4120,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>252</v>
       </c>
@@ -4062,7 +4146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>256</v>
       </c>
@@ -4088,7 +4172,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>257</v>
       </c>
@@ -4114,7 +4198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>258</v>
       </c>
@@ -4140,7 +4224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>261</v>
       </c>
@@ -4166,7 +4250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>275</v>
       </c>
@@ -4192,7 +4276,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>276</v>
       </c>
@@ -4218,7 +4302,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>263</v>
       </c>
@@ -4244,7 +4328,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>266</v>
       </c>
@@ -4270,7 +4354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>268</v>
       </c>
@@ -4296,7 +4380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>271</v>
       </c>
@@ -4322,10 +4406,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="K25" s="4"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="J27" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed the name of the zetta prefix in the 'Units_prefixes.xlsx' file.
</commit_message>
<xml_diff>
--- a/CUQ/_docs/Units_Prefixes.xlsx
+++ b/CUQ/_docs/Units_Prefixes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n00002621/PycharmProjects/SI-Reference-Point-2023/CUQ/_docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48BDB282-E8DB-F44E-9854-396DE8AF6A83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2565B5-E112-5A41-8E4B-07E084A90B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{CB28C55D-C186-8841-A70F-3B29517A5D18}"/>
   </bookViews>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="407">
   <si>
     <t>hasStartValidity</t>
   </si>
@@ -172,9 +172,6 @@
   </si>
   <si>
     <t>Y</t>
-  </si>
-  <si>
-    <t>uetta</t>
   </si>
   <si>
     <t>Z</t>
@@ -1818,10 +1815,10 @@
         <v>18</v>
       </c>
       <c r="B1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D1" t="s">
         <v>19</v>
@@ -1833,10 +1830,10 @@
         <v>2</v>
       </c>
       <c r="G1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="H1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -1856,10 +1853,10 @@
         <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -1879,10 +1876,10 @@
         <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -1902,496 +1899,496 @@
         <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>217</v>
       </c>
       <c r="B5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D5" s="1">
         <v>1E+21</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G5" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6" s="1">
         <v>1E+18</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G6" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D7" s="1">
         <v>1000000000000000</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G7" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D8" s="1">
         <v>1000000000000</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G8" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D9" s="1">
         <v>1000000000</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G9" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D10" s="1">
         <v>1000000</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G10" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D11" s="1">
         <v>1000</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G11" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D12" s="1">
         <v>100</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G12" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D13" s="1">
         <v>10</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G13" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D14" s="1">
         <v>0.1</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D15" s="1">
         <v>0.01</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D16" s="1">
         <v>1E-3</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D17" s="1">
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="H17" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D18" s="1">
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D19" s="1">
         <v>9.9999999999999998E-13</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" s="1">
         <v>1.0000000000000001E-15</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D21" s="1">
         <v>1.0000000000000001E-18</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D22" s="1">
         <v>9.9999999999999991E-22</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D23" s="1">
         <v>9.9999999999999992E-25</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F23" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D24" s="1">
         <v>1E-27</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F24" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D25" s="1">
         <v>1.0000000000000001E-30</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F25" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -2422,10 +2419,10 @@
         <v>18</v>
       </c>
       <c r="B1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s">
         <v>70</v>
-      </c>
-      <c r="C1" t="s">
-        <v>71</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>0</v>
@@ -2434,532 +2431,532 @@
         <v>1</v>
       </c>
       <c r="F1" t="s">
+        <v>71</v>
+      </c>
+      <c r="G1" t="s">
         <v>72</v>
-      </c>
-      <c r="G1" t="s">
-        <v>73</v>
       </c>
       <c r="H1" t="s">
         <v>2</v>
       </c>
       <c r="I1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J1" t="s">
         <v>15</v>
       </c>
       <c r="K1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C2" t="s">
         <v>155</v>
       </c>
-      <c r="C2" t="s">
-        <v>156</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="L2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C3" t="s">
         <v>157</v>
       </c>
-      <c r="C3" t="s">
-        <v>158</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E3"/>
       <c r="F3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H3" t="s">
         <v>13</v>
       </c>
       <c r="I3" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="L3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G4" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="L4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H5" t="s">
         <v>13</v>
       </c>
       <c r="I5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="L5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="L6" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E7"/>
       <c r="F7" t="s">
+        <v>236</v>
+      </c>
+      <c r="G7" t="s">
         <v>237</v>
-      </c>
-      <c r="G7" t="s">
-        <v>238</v>
       </c>
       <c r="H7" t="s">
         <v>13</v>
       </c>
       <c r="I7" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="J7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="K7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="L7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B8" t="s">
+        <v>167</v>
+      </c>
+      <c r="C8" t="s">
         <v>168</v>
       </c>
-      <c r="C8" t="s">
-        <v>169</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="L8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C9" t="s">
         <v>163</v>
       </c>
-      <c r="C9" t="s">
-        <v>164</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H9" t="s">
         <v>13</v>
       </c>
       <c r="I9" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="K9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="L9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B10" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" t="s">
         <v>170</v>
       </c>
-      <c r="C10" t="s">
-        <v>171</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="G10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C11" t="s">
         <v>172</v>
       </c>
-      <c r="C11" t="s">
-        <v>173</v>
-      </c>
       <c r="D11" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="F11" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="K11" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B12" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" t="s">
         <v>174</v>
       </c>
-      <c r="C12" t="s">
-        <v>175</v>
-      </c>
       <c r="D12" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G12" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K12" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L12" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B13" t="s">
+        <v>175</v>
+      </c>
+      <c r="C13" t="s">
         <v>176</v>
       </c>
-      <c r="C13" t="s">
-        <v>177</v>
-      </c>
       <c r="D13" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F13" t="s">
+        <v>232</v>
+      </c>
+      <c r="G13" t="s">
         <v>233</v>
       </c>
-      <c r="G13" t="s">
-        <v>234</v>
-      </c>
       <c r="H13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="K13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C14" t="s">
         <v>165</v>
       </c>
-      <c r="C14" t="s">
-        <v>166</v>
-      </c>
       <c r="D14" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H14" t="s">
         <v>13</v>
       </c>
       <c r="I14" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J14" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="K14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L15" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E16"/>
       <c r="F16" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="G16" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H16" t="s">
         <v>13</v>
       </c>
       <c r="I16" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="J16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L16" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
@@ -2973,25 +2970,25 @@
         <v>3</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F17" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="G17" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H17" t="s">
         <v>6</v>
       </c>
       <c r="K17" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L17" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
@@ -3005,16 +3002,16 @@
         <v>7</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F18" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G18" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H18" t="s">
         <v>10</v>
@@ -3023,10 +3020,10 @@
         <v>14</v>
       </c>
       <c r="K18" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L18" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
@@ -3040,29 +3037,29 @@
         <v>12</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E19"/>
       <c r="F19" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G19" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H19" t="s">
         <v>13</v>
       </c>
       <c r="I19" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J19" t="s">
         <v>14</v>
       </c>
       <c r="K19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L19" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -3087,7 +3084,7 @@
         <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E1" t="s">
         <v>16</v>
@@ -3095,163 +3092,163 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G3" t="s">
         <v>159</v>
-      </c>
-      <c r="G3" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G4" t="s">
         <v>161</v>
-      </c>
-      <c r="G4" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
@@ -3292,765 +3289,765 @@
         <v>18</v>
       </c>
       <c r="B1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s">
         <v>70</v>
       </c>
-      <c r="C1" t="s">
-        <v>71</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K1"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="I2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="I3" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>369</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>381</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>83</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B7" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" t="s">
-        <v>84</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C8" t="s">
-        <v>86</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="E8" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="I8" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B9" t="s">
-        <v>88</v>
-      </c>
-      <c r="C9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B10" t="s">
-        <v>90</v>
-      </c>
-      <c r="C10" t="s">
-        <v>90</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="E10" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" t="s">
+        <v>91</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B11" t="s">
-        <v>92</v>
-      </c>
-      <c r="C11" t="s">
-        <v>92</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>93</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" t="s">
-        <v>94</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>95</v>
-      </c>
       <c r="E12" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>95</v>
+      </c>
+      <c r="B13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B13" t="s">
-        <v>96</v>
-      </c>
-      <c r="C13" t="s">
-        <v>96</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" t="s">
+        <v>98</v>
+      </c>
+      <c r="C15" t="s">
+        <v>98</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B15" t="s">
-        <v>99</v>
-      </c>
-      <c r="C15" t="s">
-        <v>99</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>100</v>
-      </c>
       <c r="E15" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B16" t="s">
-        <v>101</v>
-      </c>
-      <c r="C16" t="s">
-        <v>101</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>102</v>
-      </c>
       <c r="E16" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" t="s">
+        <v>102</v>
+      </c>
+      <c r="C17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B17" t="s">
-        <v>103</v>
-      </c>
-      <c r="C17" t="s">
-        <v>103</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="E17" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B18" t="s">
-        <v>105</v>
-      </c>
-      <c r="C18" t="s">
-        <v>105</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="E18" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" t="s">
+        <v>395</v>
+      </c>
+      <c r="C19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B19" t="s">
-        <v>396</v>
-      </c>
-      <c r="C19" t="s">
-        <v>107</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="E19" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F19" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F20" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" t="s">
+        <v>109</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B21" t="s">
-        <v>110</v>
-      </c>
-      <c r="C21" t="s">
-        <v>110</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="E21" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F21" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>111</v>
+      </c>
+      <c r="B22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B22" t="s">
-        <v>112</v>
-      </c>
-      <c r="C22" t="s">
-        <v>112</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>113</v>
-      </c>
       <c r="E22" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F22" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>113</v>
+      </c>
+      <c r="B23" t="s">
+        <v>113</v>
+      </c>
+      <c r="C23" t="s">
+        <v>113</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B23" t="s">
-        <v>114</v>
-      </c>
-      <c r="C23" t="s">
-        <v>114</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>115</v>
-      </c>
       <c r="E23" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F23" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E26" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F26" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E27" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F27" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E28" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F28" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E29" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F29" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E30" s="8" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F30" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E31" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F31" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E32" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F32" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -4075,15 +4072,15 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B3">
         <v>9</v>
@@ -4091,7 +4088,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B4">
         <v>4</v>
@@ -4102,45 +4099,45 @@
         <v>18</v>
       </c>
       <c r="B6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" t="s">
         <v>70</v>
       </c>
-      <c r="C6" t="s">
-        <v>71</v>
-      </c>
       <c r="D6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" t="s">
         <v>74</v>
       </c>
-      <c r="E6" t="s">
-        <v>75</v>
-      </c>
       <c r="F6" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>251</v>
+      </c>
+      <c r="B7" t="s">
+        <v>251</v>
+      </c>
+      <c r="C7" t="s">
+        <v>251</v>
+      </c>
+      <c r="D7" t="s">
         <v>252</v>
       </c>
-      <c r="B7" t="s">
-        <v>252</v>
-      </c>
-      <c r="C7" t="s">
-        <v>252</v>
-      </c>
-      <c r="D7" t="s">
-        <v>253</v>
-      </c>
       <c r="E7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F7">
         <v>60</v>
       </c>
       <c r="G7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -4148,25 +4145,25 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F8">
         <v>3600</v>
       </c>
       <c r="G8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -4174,25 +4171,25 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F9">
         <v>86400</v>
       </c>
       <c r="G9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -4200,25 +4197,25 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>257</v>
+      </c>
+      <c r="B10" t="s">
+        <v>271</v>
+      </c>
+      <c r="C10" t="s">
         <v>258</v>
       </c>
-      <c r="B10" t="s">
-        <v>272</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>259</v>
       </c>
-      <c r="D10" t="s">
-        <v>260</v>
-      </c>
       <c r="E10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F10" s="7">
         <v>149597870700</v>
       </c>
       <c r="G10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -4226,25 +4223,25 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>260</v>
+      </c>
+      <c r="B11" t="s">
+        <v>272</v>
+      </c>
+      <c r="C11" t="s">
+        <v>260</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="B11" t="s">
-        <v>273</v>
-      </c>
-      <c r="C11" t="s">
-        <v>261</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>262</v>
-      </c>
       <c r="E11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F11" s="5">
         <v>1.7453292519943299E-2</v>
       </c>
       <c r="G11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -4252,25 +4249,25 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B12" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C12" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F12" s="5">
         <v>2.9088820866572201E-4</v>
       </c>
       <c r="G12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -4278,25 +4275,25 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>275</v>
+      </c>
+      <c r="B13" t="s">
         <v>276</v>
       </c>
-      <c r="B13" t="s">
-        <v>277</v>
-      </c>
       <c r="C13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F13" s="5">
         <v>4.8481368110953598E-6</v>
       </c>
       <c r="G13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H13">
         <v>1</v>
@@ -4304,25 +4301,25 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>262</v>
+      </c>
+      <c r="B14" t="s">
+        <v>262</v>
+      </c>
+      <c r="C14" t="s">
+        <v>262</v>
+      </c>
+      <c r="D14" t="s">
         <v>263</v>
       </c>
-      <c r="B14" t="s">
-        <v>263</v>
-      </c>
-      <c r="C14" t="s">
-        <v>263</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>264</v>
-      </c>
-      <c r="E14" t="s">
-        <v>265</v>
       </c>
       <c r="F14">
         <v>1E-3</v>
       </c>
       <c r="G14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H14">
         <v>3</v>
@@ -4330,25 +4327,25 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>265</v>
+      </c>
+      <c r="B15" t="s">
+        <v>265</v>
+      </c>
+      <c r="C15" t="s">
+        <v>265</v>
+      </c>
+      <c r="D15" t="s">
         <v>266</v>
       </c>
-      <c r="B15" t="s">
-        <v>266</v>
-      </c>
-      <c r="C15" t="s">
-        <v>266</v>
-      </c>
-      <c r="D15" t="s">
-        <v>267</v>
-      </c>
       <c r="E15" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F15">
         <v>1000</v>
       </c>
       <c r="G15" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -4356,25 +4353,25 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B16" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C16" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D16" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E16" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F16" s="6">
         <v>1.6605390666E-27</v>
       </c>
       <c r="G16" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -4382,25 +4379,25 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B17" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C17" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D17" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F17" s="7">
         <v>1.6021766339999999E-19</v>
       </c>
       <c r="G17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H17">
         <v>1</v>

</xml_diff>